<commit_message>
got precision up to 97% and recall to 78% with this prompt
</commit_message>
<xml_diff>
--- a/output/alt_abbrev_annotation_wo_context_df.xlsx
+++ b/output/alt_abbrev_annotation_wo_context_df.xlsx
@@ -2831,7 +2831,7 @@
         </is>
       </c>
       <c r="H61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -4118,7 +4118,7 @@
         </is>
       </c>
       <c r="H94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="H165" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I165" t="inlineStr">
         <is>
@@ -8708,7 +8708,7 @@
         </is>
       </c>
       <c r="H210" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I210" t="inlineStr">
         <is>
@@ -9697,7 +9697,7 @@
         </is>
       </c>
       <c r="H233" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I233" t="inlineStr">
         <is>
@@ -10213,7 +10213,7 @@
         </is>
       </c>
       <c r="H245" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I245" t="inlineStr">
         <is>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="H246" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I246" t="inlineStr">
         <is>
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="H274" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I274" t="inlineStr">
         <is>
@@ -14599,7 +14599,7 @@
         </is>
       </c>
       <c r="H347" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I347" t="inlineStr">
         <is>
@@ -15158,7 +15158,7 @@
         </is>
       </c>
       <c r="H360" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I360" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
adding a judge prompt after seems to decrease recall and precision. I tried both ways of placing the simple prompt as the first prompt and as the judge prompt and each time the accuracy was affected negatively
</commit_message>
<xml_diff>
--- a/output/alt_abbrev_annotation_wo_context_df.xlsx
+++ b/output/alt_abbrev_annotation_wo_context_df.xlsx
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="H17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="H111" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="H134" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="H165" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I165" t="inlineStr">
         <is>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="H187" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I187" t="inlineStr">
         <is>
@@ -10213,7 +10213,7 @@
         </is>
       </c>
       <c r="H245" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I245" t="inlineStr">
         <is>
@@ -14986,7 +14986,7 @@
         </is>
       </c>
       <c r="H356" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I356" t="inlineStr">
         <is>

</xml_diff>